<commit_message>
tprm demo: regenerate synthetic assessments from approved-rule run (seals 4556/4561, all provenance VERIFIED, blocked_pending_sme)
</commit_message>
<xml_diff>
--- a/public/demo/EVE_TPRM_Workpaper_SyntheticVendorA.xlsx
+++ b/public/demo/EVE_TPRM_Workpaper_SyntheticVendorA.xlsx
@@ -708,7 +708,7 @@
       <c r="D11" s="8" t="n"/>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>EVE-TPRM-00004516</t>
+          <t>EVE-TPRM-00004556</t>
         </is>
       </c>
       <c r="F11" s="8" t="n"/>
@@ -783,7 +783,7 @@
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="15" t="n">
@@ -791,7 +791,7 @@
       </c>
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F19" s="8" t="n"/>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
-          <t>assess_3ef8282a</t>
+          <t>assess_9757896f</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>EVE-TPRM-00004516</t>
+          <t>EVE-TPRM-00004556</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="C37" s="20" t="inlineStr">
         <is>
-          <t>2026-06-12 22:49 UTC</t>
+          <t>2026-06-13 08:26 UTC</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="L2" s="25" t="inlineStr">
         <is>
-          <t>EVE-TPRM-00004512</t>
+          <t>EVE-TPRM-00004552</t>
         </is>
       </c>
     </row>
@@ -1240,12 +1240,12 @@
       </c>
       <c r="I3" s="23" t="inlineStr">
         <is>
-          <t>NO_ANSWER</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="J3" s="23" t="inlineStr">
         <is>
-          <t>unavailable</t>
+          <t>blocked_pending_sme</t>
         </is>
       </c>
       <c r="K3" s="23" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="L3" s="25" t="inlineStr">
         <is>
-          <t>EVE-TPRM-00004513</t>
+          <t>EVE-TPRM-00004553</t>
         </is>
       </c>
     </row>
@@ -1302,12 +1302,12 @@
       </c>
       <c r="I4" s="23" t="inlineStr">
         <is>
-          <t>NO_ANSWER</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="J4" s="23" t="inlineStr">
         <is>
-          <t>unavailable</t>
+          <t>blocked_pending_sme</t>
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="L4" s="25" t="inlineStr">
         <is>
-          <t>EVE-TPRM-00004514</t>
+          <t>EVE-TPRM-00004554</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="I5" s="23" t="inlineStr">
         <is>
-          <t>NO_ANSWER</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="J5" s="23" t="inlineStr">
         <is>
-          <t>unavailable</t>
+          <t>blocked_pending_sme</t>
         </is>
       </c>
       <c r="K5" s="23" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="L5" s="25" t="inlineStr">
         <is>
-          <t>EVE-TPRM-00004515</t>
+          <t>EVE-TPRM-00004555</t>
         </is>
       </c>
     </row>
@@ -6885,28 +6885,44 @@
       </c>
       <c r="D3" s="23" t="inlineStr">
         <is>
-          <t>NO_ANSWER</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E3" s="23" t="inlineStr">
         <is>
-          <t>unavailable</t>
-        </is>
-      </c>
-      <c r="F3" s="23" t="inlineStr"/>
-      <c r="G3" s="23" t="inlineStr"/>
-      <c r="H3" s="20" t="inlineStr"/>
-      <c r="I3" s="23" t="inlineStr"/>
-      <c r="J3" s="23" t="inlineStr"/>
+          <t>blocked_pending_sme</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>EVE-2026-000010</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr">
+        <is>
+          <t>EVEV-COMP-20260613-000001</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>4ac30772a825f711d384642d9c5d65a48906deb7a0a8174556dc78e20c3c2f0a</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" s="23" t="inlineStr">
+        <is>
+          <t>joakim</t>
+        </is>
+      </c>
       <c r="K3" s="23" t="inlineStr"/>
       <c r="L3" s="23" t="inlineStr"/>
       <c r="M3" s="23" t="inlineStr"/>
       <c r="N3" s="20" t="inlineStr"/>
-      <c r="O3" s="20" t="inlineStr">
-        <is>
-          <t>NO_APPROVED_RULE_LINEAGE</t>
-        </is>
-      </c>
+      <c r="O3" s="20" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
@@ -6926,28 +6942,44 @@
       </c>
       <c r="D4" s="23" t="inlineStr">
         <is>
-          <t>NO_ANSWER</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
-          <t>unavailable</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr"/>
-      <c r="G4" s="23" t="inlineStr"/>
-      <c r="H4" s="20" t="inlineStr"/>
-      <c r="I4" s="23" t="inlineStr"/>
-      <c r="J4" s="23" t="inlineStr"/>
+          <t>blocked_pending_sme</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>EVE-2026-000011</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>EVEV-COMP-20260613-000002</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>9ce5b2abce09d3ec0569849e17653821c0d3462652f18b846ed06ff4d01ed1bf</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr">
+        <is>
+          <t>joakim</t>
+        </is>
+      </c>
       <c r="K4" s="23" t="inlineStr"/>
       <c r="L4" s="23" t="inlineStr"/>
       <c r="M4" s="23" t="inlineStr"/>
       <c r="N4" s="20" t="inlineStr"/>
-      <c r="O4" s="20" t="inlineStr">
-        <is>
-          <t>NO_APPROVED_RULE_LINEAGE</t>
-        </is>
-      </c>
+      <c r="O4" s="20" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
@@ -6967,28 +6999,44 @@
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>NO_ANSWER</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E5" s="23" t="inlineStr">
         <is>
-          <t>unavailable</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="inlineStr"/>
-      <c r="G5" s="23" t="inlineStr"/>
-      <c r="H5" s="20" t="inlineStr"/>
-      <c r="I5" s="23" t="inlineStr"/>
-      <c r="J5" s="23" t="inlineStr"/>
+          <t>blocked_pending_sme</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>EVE-2026-000012</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>EVEV-COMP-20260613-000003</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>1e7718f74fa6ce46f4292d35bc9ec57f3b601f3ac30bc6ccc420730da3687d75</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr">
+        <is>
+          <t>joakim</t>
+        </is>
+      </c>
       <c r="K5" s="23" t="inlineStr"/>
       <c r="L5" s="23" t="inlineStr"/>
       <c r="M5" s="23" t="inlineStr"/>
       <c r="N5" s="20" t="inlineStr"/>
-      <c r="O5" s="20" t="inlineStr">
-        <is>
-          <t>NO_APPROVED_RULE_LINEAGE</t>
-        </is>
-      </c>
+      <c r="O5" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O5"/>

</xml_diff>